<commit_message>
add updated lag selection files
</commit_message>
<xml_diff>
--- a/results/lag_selection_results.xlsx
+++ b/results/lag_selection_results.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,218 +413,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>lag_y</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>lag_NASCDI_pos</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>lag_NASCDI_neg</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>AIC</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>BIC</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>HQIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>weekly_model_Shopian_American_A_posneg.csv</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>weekly_model_Shopian_American_B_posneg.csv</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>weekly_model_Shopian_Delicious_A_posneg.csv</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>weekly_model_Shopian_Delicious_B_posneg.csv</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>weekly_model_Sopore_American_A_posneg.csv</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>weekly_model_Sopore_American_B_posneg.csv</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>weekly_model_Sopore_Delicious_A_posneg.csv</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>weekly_model_Sopore_Delicious_B_posneg.csv</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>weekly_prices_all_posneg.csv</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added modified NARDL lag selection
</commit_message>
<xml_diff>
--- a/results/lag_selection_results.xlsx
+++ b/results/lag_selection_results.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +425,302 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>lag_y</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>lag_NASCDI_pos</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>lag_NASCDI_neg</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>AIC</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>BIC</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>HQIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>weekly_model_Shopian_American_A_posneg.csv</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>[0, 1]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>[0]</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>-133.1414</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-119.157</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-127.5526</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>weekly_model_Shopian_American_B_posneg.csv</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[0, 1]</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>[0]</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>-79.8219</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-65.83750000000001</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-74.23309999999999</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>weekly_model_Shopian_Delicious_A_posneg.csv</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>[0, 1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>[0, 1, 2]</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>-241.7947</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-203.8613</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-226.4063</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>weekly_model_Shopian_Delicious_B_posneg.csv</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>[0, 1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>[0, 1, 2]</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>-144.2958</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-114.1977</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-132.0807</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>weekly_model_Sopore_American_A_posneg.csv</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>[0, 1]</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>-446.8965</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-430.3059</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-440.1853</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>weekly_model_Sopore_American_B_posneg.csv</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[0]</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-318.4099</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-305.1374</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-313.0409</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>weekly_model_Sopore_Delicious_A_posneg.csv</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>[0, 1]</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>[0]</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>-506.4543</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-485.5705</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-498.0397</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>weekly_model_Sopore_Delicious_B_posneg.csv</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>[0, 1]</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>-323.6317</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-306.2285</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-316.6195</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>weekly_prices_all_posneg.csv</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[0]</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>[0, 1, 2]</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>-1727.2471</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-1691.1922</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-1713.7061</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>